<commit_message>
Update READMEs and institutional briefs
</commit_message>
<xml_diff>
--- a/output/summary_tables/Biennial Report 2001 Summary Tables.xlsx
+++ b/output/summary_tables/Biennial Report 2001 Summary Tables.xlsx
@@ -1922,11 +1922,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="28.5"/>
-    <col min="2" max="7" bestFit="1" customWidth="1" hidden="false" width="12.664"/>
+    <col min="2" max="9" bestFit="1" customWidth="1" hidden="false" width="12.664"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1965,6 +1965,16 @@
           <t>No %</t>
         </is>
       </c>
+      <c r="H1" s="23" t="inlineStr">
+        <is>
+          <t>Unknown N</t>
+        </is>
+      </c>
+      <c r="I1" s="23" t="inlineStr">
+        <is>
+          <t>Unknown %</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1990,6 +2000,12 @@
       <c r="G2" s="10">
         <v>12.27</v>
       </c>
+      <c r="H2" s="10">
+        <v>0</v>
+      </c>
+      <c r="I2" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -2015,6 +2031,12 @@
       <c r="G3" s="10">
         <v>79.86</v>
       </c>
+      <c r="H3" s="10">
+        <v>0</v>
+      </c>
+      <c r="I3" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2040,6 +2062,12 @@
       <c r="G4" s="10">
         <v>14.41</v>
       </c>
+      <c r="H4" s="10">
+        <v>0</v>
+      </c>
+      <c r="I4" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -2065,6 +2093,12 @@
       <c r="G5" s="10">
         <v>58.56</v>
       </c>
+      <c r="H5" s="10">
+        <v>0</v>
+      </c>
+      <c r="I5" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -2090,6 +2124,12 @@
       <c r="G6" s="10">
         <v>3.1</v>
       </c>
+      <c r="H6" s="10">
+        <v>0</v>
+      </c>
+      <c r="I6" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -2115,6 +2155,12 @@
       <c r="G7" s="10">
         <v>77.66</v>
       </c>
+      <c r="H7" s="10">
+        <v>0</v>
+      </c>
+      <c r="I7" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -2140,6 +2186,12 @@
       <c r="G8" s="10">
         <v>17.29</v>
       </c>
+      <c r="H8" s="10">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -2165,6 +2217,12 @@
       <c r="G9" s="10">
         <v>26.43</v>
       </c>
+      <c r="H9" s="10">
+        <v>0</v>
+      </c>
+      <c r="I9" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -2190,6 +2248,12 @@
       <c r="G10" s="10">
         <v>1.15</v>
       </c>
+      <c r="H10" s="10">
+        <v>0</v>
+      </c>
+      <c r="I10" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -2215,6 +2279,12 @@
       <c r="G11" s="10">
         <v>88.38</v>
       </c>
+      <c r="H11" s="10">
+        <v>0</v>
+      </c>
+      <c r="I11" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -2239,6 +2309,12 @@
       </c>
       <c r="G12" s="10">
         <v>78.61</v>
+      </c>
+      <c r="H12" s="10">
+        <v>0</v>
+      </c>
+      <c r="I12" s="10">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>